<commit_message>
Improve test coverage for formula behaviors. Handle some edge cases where formulas return empty strings.
</commit_message>
<xml_diff>
--- a/source/Sylvan.Data.Excel.Tests/Data/SharedFormulaString.xlsx
+++ b/source/Sylvan.Data.Excel.Tests/Data/SharedFormulaString.xlsx
@@ -1,38 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BRANDO~1\AppData\Local\Temp\claude\c--Users-BrandonWinsley-source-repos-Sylvan-Data-Excel\56a208d4-bc0c-4e39-b734-32db3cefd70a\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\markp\source\Sylvan.Data.Excel\source\Sylvan.Data.Excel.Tests\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{729AE3DA-76BC-4DF7-871B-C1C200211B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B3A62B-8A5A-41BA-A610-571734EBDDC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{CEEE9DCE-D56E-475F-B7E1-340EAEE93589}"/>
+    <workbookView xWindow="1272" yWindow="3600" windowWidth="25428" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -44,7 +30,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -99,39 +85,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -164,26 +150,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -216,23 +185,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -294,6 +246,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -302,13 +261,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -373,102 +325,166 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59AC6C35-1026-437B-9D27-EE1795B6011E}">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" t="str">
         <f>"Item "&amp;A1</f>
-        <v>Item 1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 0</v>
+      </c>
+      <c r="C1">
+        <f>A1+100</f>
+        <v>100</v>
+      </c>
+      <c r="D1" t="b">
+        <f>MOD(A1,2)=1</f>
+        <v>0</v>
+      </c>
+      <c r="E1" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B7" si="0">"Item "&amp;A2</f>
-        <v>Item 2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 1</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C7" si="1">A2+100</f>
+        <v>101</v>
+      </c>
+      <c r="D2" t="b">
+        <f t="shared" ref="D2:D7" si="2">MOD(A2,2)=1</f>
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
-        <v>Item 3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 2</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="1"/>
+        <v>102</v>
+      </c>
+      <c r="D3" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E3" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>Item 4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 3</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="1"/>
+        <v>103</v>
+      </c>
+      <c r="D4" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v>Item 5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 4</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="1"/>
+        <v>104</v>
+      </c>
+      <c r="D5" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E5" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
-        <v>Item 6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>Item 5</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+      <c r="D6" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="E6" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
-        <v>Item 7</v>
+        <v>Item 6</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="1"/>
+        <v>106</v>
+      </c>
+      <c r="D7" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E7" t="str">
+        <f>""</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>